<commit_message>
Test protocol workbook: summary counts per language sheet only.
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/LifeThreads_Test_Protocol_build24.xlsx
+++ b/docs/LifeThreads_Test_Protocol_build24.xlsx
@@ -517,14 +517,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E15"/>
+  <dimension ref="A1:D15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="16" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -603,11 +602,6 @@
           <t>العربية</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -627,10 +621,6 @@
         <f>ROWS('العربية'!G2:G47)</f>
         <v/>
       </c>
-      <c r="E8">
-        <f>B8</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -650,10 +640,6 @@
         <f>COUNTIF('العربية'!G2:G47,"ناجح")</f>
         <v/>
       </c>
-      <c r="E9">
-        <f>SUM(B9:D9)</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -673,10 +659,6 @@
         <f>COUNTIF('العربية'!G2:G47,"خطأ")</f>
         <v/>
       </c>
-      <c r="E10">
-        <f>SUM(B10:D10)</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -696,10 +678,6 @@
         <f>COUNTIF('العربية'!G2:G47,"متعذّر")</f>
         <v/>
       </c>
-      <c r="E11">
-        <f>SUM(B11:D11)</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -719,10 +697,6 @@
         <f>COUNTIF('العربية'!G2:G47,"لا ينطبق")</f>
         <v/>
       </c>
-      <c r="E12">
-        <f>SUM(B12:D12)</f>
-        <v/>
-      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -740,10 +714,6 @@
       </c>
       <c r="D13">
         <f>COUNTBLANK('العربية'!G2:G47)</f>
-        <v/>
-      </c>
-      <c r="E13">
-        <f>SUM(B13:D13)</f>
         <v/>
       </c>
     </row>

</xml_diff>